<commit_message>
Mise à jour des projections des banques centrales (2026-09-18)
</commit_message>
<xml_diff>
--- a/data/boe/boe_mpr.xlsx
+++ b/data/boe/boe_mpr.xlsx
@@ -524,11 +524,11 @@
     <col width="10" customWidth="1" min="52" max="52"/>
     <col width="10" customWidth="1" min="53" max="53"/>
     <col width="17" customWidth="1" min="54" max="54"/>
-    <col width="10" customWidth="1" min="55" max="55"/>
-    <col width="10" customWidth="1" min="56" max="56"/>
-    <col width="10" customWidth="1" min="57" max="57"/>
-    <col width="10" customWidth="1" min="58" max="58"/>
-    <col width="10" customWidth="1" min="59" max="59"/>
+    <col width="11" customWidth="1" min="55" max="55"/>
+    <col width="11" customWidth="1" min="56" max="56"/>
+    <col width="11" customWidth="1" min="57" max="57"/>
+    <col width="11" customWidth="1" min="58" max="58"/>
+    <col width="11" customWidth="1" min="59" max="59"/>
     <col width="11" customWidth="1" min="60" max="60"/>
     <col width="11" customWidth="1" min="61" max="61"/>
     <col width="11" customWidth="1" min="62" max="62"/>
@@ -550,26 +550,26 @@
     <col width="10" customWidth="1" min="78" max="78"/>
     <col width="10" customWidth="1" min="79" max="79"/>
     <col width="21" customWidth="1" min="80" max="80"/>
-    <col width="10" customWidth="1" min="81" max="81"/>
+    <col width="13" customWidth="1" min="81" max="81"/>
     <col width="14" customWidth="1" min="82" max="82"/>
     <col width="11" customWidth="1" min="83" max="83"/>
     <col width="14" customWidth="1" min="84" max="84"/>
-    <col width="10" customWidth="1" min="85" max="85"/>
-    <col width="10" customWidth="1" min="86" max="86"/>
+    <col width="14" customWidth="1" min="85" max="85"/>
+    <col width="13" customWidth="1" min="86" max="86"/>
     <col width="15" customWidth="1" min="87" max="87"/>
     <col width="15" customWidth="1" min="88" max="88"/>
     <col width="14" customWidth="1" min="89" max="89"/>
     <col width="15" customWidth="1" min="90" max="90"/>
     <col width="11" customWidth="1" min="91" max="91"/>
     <col width="15" customWidth="1" min="92" max="92"/>
-    <col width="10" customWidth="1" min="93" max="93"/>
-    <col width="13" customWidth="1" min="94" max="94"/>
+    <col width="12" customWidth="1" min="93" max="93"/>
+    <col width="15" customWidth="1" min="94" max="94"/>
     <col width="14" customWidth="1" min="95" max="95"/>
-    <col width="10" customWidth="1" min="96" max="96"/>
-    <col width="11" customWidth="1" min="97" max="97"/>
+    <col width="12" customWidth="1" min="96" max="96"/>
+    <col width="15" customWidth="1" min="97" max="97"/>
     <col width="13" customWidth="1" min="98" max="98"/>
     <col width="14" customWidth="1" min="99" max="99"/>
-    <col width="11" customWidth="1" min="100" max="100"/>
+    <col width="10" customWidth="1" min="100" max="100"/>
     <col width="10" customWidth="1" min="101" max="101"/>
     <col width="13" customWidth="1" min="102" max="102"/>
     <col width="13" customWidth="1" min="103" max="103"/>
@@ -1377,19 +1377,35 @@
       <c r="AY3" s="3" t="inlineStr"/>
       <c r="AZ3" s="3" t="inlineStr"/>
       <c r="BA3" s="3" t="inlineStr"/>
-      <c r="BB3" s="3" t="inlineStr"/>
+      <c r="BB3" s="3" t="inlineStr">
+        <is>
+          <t>3.6 (3.9)</t>
+        </is>
+      </c>
       <c r="BC3" s="3" t="inlineStr"/>
       <c r="BD3" s="3" t="inlineStr"/>
       <c r="BE3" s="3" t="inlineStr"/>
-      <c r="BF3" s="3" t="inlineStr"/>
+      <c r="BF3" s="3" t="inlineStr">
+        <is>
+          <t>3.9 (4.4)</t>
+        </is>
+      </c>
       <c r="BG3" s="3" t="inlineStr"/>
       <c r="BH3" s="3" t="inlineStr"/>
       <c r="BI3" s="3" t="inlineStr"/>
-      <c r="BJ3" s="3" t="inlineStr"/>
+      <c r="BJ3" s="3" t="inlineStr">
+        <is>
+          <t>4.6 (4.7)</t>
+        </is>
+      </c>
       <c r="BK3" s="3" t="inlineStr"/>
       <c r="BL3" s="3" t="inlineStr"/>
       <c r="BM3" s="3" t="inlineStr"/>
-      <c r="BN3" s="3" t="inlineStr"/>
+      <c r="BN3" s="3" t="inlineStr">
+        <is>
+          <t>5.5</t>
+        </is>
+      </c>
       <c r="BO3" s="3" t="inlineStr"/>
       <c r="BP3" s="3" t="inlineStr"/>
       <c r="BQ3" s="3" t="inlineStr"/>
@@ -1413,7 +1429,7 @@
       <c r="CE3" s="3" t="inlineStr"/>
       <c r="CF3" s="3" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>-1.25 (-0.5)</t>
         </is>
       </c>
       <c r="CG3" s="3" t="inlineStr"/>
@@ -1421,7 +1437,7 @@
       <c r="CI3" s="3" t="inlineStr"/>
       <c r="CJ3" s="3" t="inlineStr">
         <is>
-          <t>0.25 (-0.5)</t>
+          <t>-1.75 (-0.5)</t>
         </is>
       </c>
       <c r="CK3" s="3" t="inlineStr"/>
@@ -1429,7 +1445,7 @@
       <c r="CM3" s="3" t="inlineStr"/>
       <c r="CN3" s="3" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>-2.25</t>
         </is>
       </c>
       <c r="CO3" s="3" t="inlineStr"/>
@@ -1579,19 +1595,35 @@
       <c r="AZ4" s="3" t="inlineStr"/>
       <c r="BA4" s="3" t="inlineStr"/>
       <c r="BB4" s="3" t="inlineStr"/>
-      <c r="BC4" s="3" t="inlineStr"/>
+      <c r="BC4" s="3" t="inlineStr">
+        <is>
+          <t>3.7 (3.5)</t>
+        </is>
+      </c>
       <c r="BD4" s="3" t="inlineStr"/>
       <c r="BE4" s="3" t="inlineStr"/>
       <c r="BF4" s="3" t="inlineStr"/>
-      <c r="BG4" s="3" t="inlineStr"/>
+      <c r="BG4" s="3" t="inlineStr">
+        <is>
+          <t>4.4 (4.1)</t>
+        </is>
+      </c>
       <c r="BH4" s="3" t="inlineStr"/>
       <c r="BI4" s="3" t="inlineStr"/>
       <c r="BJ4" s="3" t="inlineStr"/>
-      <c r="BK4" s="3" t="inlineStr"/>
+      <c r="BK4" s="3" t="inlineStr">
+        <is>
+          <t>5.5 (4.8)</t>
+        </is>
+      </c>
       <c r="BL4" s="3" t="inlineStr"/>
       <c r="BM4" s="3" t="inlineStr"/>
       <c r="BN4" s="3" t="inlineStr"/>
-      <c r="BO4" s="3" t="inlineStr"/>
+      <c r="BO4" s="3" t="inlineStr">
+        <is>
+          <t>6.3</t>
+        </is>
+      </c>
       <c r="BP4" s="3" t="inlineStr"/>
       <c r="BQ4" s="3" t="inlineStr"/>
       <c r="BR4" s="3" t="inlineStr"/>
@@ -1607,7 +1639,7 @@
       <c r="CB4" s="3" t="inlineStr"/>
       <c r="CC4" s="3" t="inlineStr">
         <is>
-          <t>0.75</t>
+          <t>0.75 (0.25)</t>
         </is>
       </c>
       <c r="CD4" s="3" t="inlineStr"/>
@@ -1615,7 +1647,7 @@
       <c r="CF4" s="3" t="inlineStr"/>
       <c r="CG4" s="3" t="inlineStr">
         <is>
-          <t>0.25</t>
+          <t>-2.25 (-1.5)</t>
         </is>
       </c>
       <c r="CH4" s="3" t="inlineStr"/>
@@ -1623,7 +1655,7 @@
       <c r="CJ4" s="3" t="inlineStr"/>
       <c r="CK4" s="3" t="inlineStr">
         <is>
-          <t>-2</t>
+          <t>-3.25 (-2)</t>
         </is>
       </c>
       <c r="CL4" s="3" t="inlineStr"/>
@@ -1631,7 +1663,7 @@
       <c r="CN4" s="3" t="inlineStr"/>
       <c r="CO4" s="3" t="inlineStr">
         <is>
-          <t>0.25</t>
+          <t>-3.75</t>
         </is>
       </c>
       <c r="CP4" s="3" t="inlineStr"/>
@@ -1781,19 +1813,35 @@
       <c r="BA5" s="3" t="inlineStr"/>
       <c r="BB5" s="3" t="inlineStr"/>
       <c r="BC5" s="3" t="inlineStr"/>
-      <c r="BD5" s="3" t="inlineStr"/>
+      <c r="BD5" s="3" t="inlineStr">
+        <is>
+          <t>3.7 (3.7)</t>
+        </is>
+      </c>
       <c r="BE5" s="3" t="inlineStr"/>
       <c r="BF5" s="3" t="inlineStr"/>
       <c r="BG5" s="3" t="inlineStr"/>
-      <c r="BH5" s="3" t="inlineStr"/>
+      <c r="BH5" s="3" t="inlineStr">
+        <is>
+          <t>4.9 (4.7)</t>
+        </is>
+      </c>
       <c r="BI5" s="3" t="inlineStr"/>
       <c r="BJ5" s="3" t="inlineStr"/>
       <c r="BK5" s="3" t="inlineStr"/>
-      <c r="BL5" s="3" t="inlineStr"/>
+      <c r="BL5" s="3" t="inlineStr">
+        <is>
+          <t>5.9 (5.7)</t>
+        </is>
+      </c>
       <c r="BM5" s="3" t="inlineStr"/>
       <c r="BN5" s="3" t="inlineStr"/>
       <c r="BO5" s="3" t="inlineStr"/>
-      <c r="BP5" s="3" t="inlineStr"/>
+      <c r="BP5" s="3" t="inlineStr">
+        <is>
+          <t>6.4</t>
+        </is>
+      </c>
       <c r="BQ5" s="3" t="inlineStr"/>
       <c r="BR5" s="3" t="inlineStr"/>
       <c r="BS5" s="3" t="inlineStr"/>
@@ -1817,7 +1865,7 @@
       <c r="CG5" s="3" t="inlineStr"/>
       <c r="CH5" s="3" t="inlineStr">
         <is>
-          <t>-2</t>
+          <t>-2.5 (-2.5)</t>
         </is>
       </c>
       <c r="CI5" s="3" t="inlineStr"/>
@@ -1825,7 +1873,7 @@
       <c r="CK5" s="3" t="inlineStr"/>
       <c r="CL5" s="3" t="inlineStr">
         <is>
-          <t>0.5</t>
+          <t>-3 (-3.25)</t>
         </is>
       </c>
       <c r="CM5" s="3" t="inlineStr"/>
@@ -1833,7 +1881,7 @@
       <c r="CO5" s="3" t="inlineStr"/>
       <c r="CP5" s="3" t="inlineStr">
         <is>
-          <t>-2</t>
+          <t>-3</t>
         </is>
       </c>
       <c r="CQ5" s="3" t="inlineStr"/>
@@ -1983,19 +2031,35 @@
       <c r="BB6" s="3" t="inlineStr"/>
       <c r="BC6" s="3" t="inlineStr"/>
       <c r="BD6" s="3" t="inlineStr"/>
-      <c r="BE6" s="3" t="inlineStr"/>
+      <c r="BE6" s="3" t="inlineStr">
+        <is>
+          <t>3.8 (3.8)</t>
+        </is>
+      </c>
       <c r="BF6" s="3" t="inlineStr"/>
       <c r="BG6" s="3" t="inlineStr"/>
       <c r="BH6" s="3" t="inlineStr"/>
-      <c r="BI6" s="3" t="inlineStr"/>
+      <c r="BI6" s="3" t="inlineStr">
+        <is>
+          <t>4.4 (5.2)</t>
+        </is>
+      </c>
       <c r="BJ6" s="3" t="inlineStr"/>
       <c r="BK6" s="3" t="inlineStr"/>
       <c r="BL6" s="3" t="inlineStr"/>
-      <c r="BM6" s="3" t="inlineStr"/>
+      <c r="BM6" s="3" t="inlineStr">
+        <is>
+          <t>5.0 (6.0)</t>
+        </is>
+      </c>
       <c r="BN6" s="3" t="inlineStr"/>
       <c r="BO6" s="3" t="inlineStr"/>
       <c r="BP6" s="3" t="inlineStr"/>
-      <c r="BQ6" s="3" t="inlineStr"/>
+      <c r="BQ6" s="3" t="inlineStr">
+        <is>
+          <t>5.3</t>
+        </is>
+      </c>
       <c r="BR6" s="3" t="inlineStr"/>
       <c r="BS6" s="3" t="inlineStr"/>
       <c r="BT6" s="3" t="inlineStr"/>
@@ -2019,7 +2083,7 @@
       <c r="CH6" s="3" t="inlineStr"/>
       <c r="CI6" s="3" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>-1.5 (-2.5)</t>
         </is>
       </c>
       <c r="CJ6" s="3" t="inlineStr"/>
@@ -2027,7 +2091,7 @@
       <c r="CL6" s="3" t="inlineStr"/>
       <c r="CM6" s="3" t="inlineStr">
         <is>
-          <t>0.5</t>
+          <t>-2 (-3)</t>
         </is>
       </c>
       <c r="CN6" s="3" t="inlineStr"/>
@@ -2185,19 +2249,35 @@
       <c r="BC7" s="3" t="inlineStr"/>
       <c r="BD7" s="3" t="inlineStr"/>
       <c r="BE7" s="3" t="inlineStr"/>
-      <c r="BF7" s="3" t="inlineStr"/>
+      <c r="BF7" s="3" t="inlineStr">
+        <is>
+          <t>3.8 (4.1)</t>
+        </is>
+      </c>
       <c r="BG7" s="3" t="inlineStr"/>
       <c r="BH7" s="3" t="inlineStr"/>
       <c r="BI7" s="3" t="inlineStr"/>
-      <c r="BJ7" s="3" t="inlineStr"/>
+      <c r="BJ7" s="3" t="inlineStr">
+        <is>
+          <t>3.9 (4.6)</t>
+        </is>
+      </c>
       <c r="BK7" s="3" t="inlineStr"/>
       <c r="BL7" s="3" t="inlineStr"/>
       <c r="BM7" s="3" t="inlineStr"/>
-      <c r="BN7" s="3" t="inlineStr"/>
+      <c r="BN7" s="3" t="inlineStr">
+        <is>
+          <t>4.3 (5.1)</t>
+        </is>
+      </c>
       <c r="BO7" s="3" t="inlineStr"/>
       <c r="BP7" s="3" t="inlineStr"/>
       <c r="BQ7" s="3" t="inlineStr"/>
-      <c r="BR7" s="3" t="inlineStr"/>
+      <c r="BR7" s="3" t="inlineStr">
+        <is>
+          <t>4.5</t>
+        </is>
+      </c>
       <c r="BS7" s="3" t="inlineStr"/>
       <c r="BT7" s="3" t="inlineStr"/>
       <c r="BU7" s="3" t="inlineStr"/>
@@ -2221,7 +2301,7 @@
       <c r="CI7" s="3" t="inlineStr"/>
       <c r="CJ7" s="3" t="inlineStr">
         <is>
-          <t>-0.5</t>
+          <t>-0.5 (-1.75)</t>
         </is>
       </c>
       <c r="CK7" s="3" t="inlineStr"/>
@@ -2229,7 +2309,7 @@
       <c r="CM7" s="3" t="inlineStr"/>
       <c r="CN7" s="3" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>-1 (-2.25)</t>
         </is>
       </c>
       <c r="CO7" s="3" t="inlineStr"/>
@@ -2237,7 +2317,7 @@
       <c r="CQ7" s="3" t="inlineStr"/>
       <c r="CR7" s="3" t="inlineStr">
         <is>
-          <t>0.75</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="CS7" s="3" t="inlineStr"/>
@@ -2387,19 +2467,35 @@
       <c r="BD8" s="3" t="inlineStr"/>
       <c r="BE8" s="3" t="inlineStr"/>
       <c r="BF8" s="3" t="inlineStr"/>
-      <c r="BG8" s="3" t="inlineStr"/>
+      <c r="BG8" s="3" t="inlineStr">
+        <is>
+          <t>4.1 (3.8)</t>
+        </is>
+      </c>
       <c r="BH8" s="3" t="inlineStr"/>
       <c r="BI8" s="3" t="inlineStr"/>
       <c r="BJ8" s="3" t="inlineStr"/>
-      <c r="BK8" s="3" t="inlineStr"/>
+      <c r="BK8" s="3" t="inlineStr">
+        <is>
+          <t>4.3 (3.9)</t>
+        </is>
+      </c>
       <c r="BL8" s="3" t="inlineStr"/>
       <c r="BM8" s="3" t="inlineStr"/>
       <c r="BN8" s="3" t="inlineStr"/>
-      <c r="BO8" s="3" t="inlineStr"/>
+      <c r="BO8" s="3" t="inlineStr">
+        <is>
+          <t>4.8 (4.4)</t>
+        </is>
+      </c>
       <c r="BP8" s="3" t="inlineStr"/>
       <c r="BQ8" s="3" t="inlineStr"/>
       <c r="BR8" s="3" t="inlineStr"/>
-      <c r="BS8" s="3" t="inlineStr"/>
+      <c r="BS8" s="3" t="inlineStr">
+        <is>
+          <t>4.8</t>
+        </is>
+      </c>
       <c r="BT8" s="3" t="inlineStr"/>
       <c r="BU8" s="3" t="inlineStr"/>
       <c r="BV8" s="3" t="inlineStr"/>
@@ -2431,7 +2527,7 @@
       <c r="CN8" s="3" t="inlineStr"/>
       <c r="CO8" s="3" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>-1.25 (-1)</t>
         </is>
       </c>
       <c r="CP8" s="3" t="inlineStr"/>
@@ -2439,7 +2535,7 @@
       <c r="CR8" s="3" t="inlineStr"/>
       <c r="CS8" s="3" t="inlineStr">
         <is>
-          <t>0.25 (-1)</t>
+          <t>-1.5</t>
         </is>
       </c>
       <c r="CT8" s="3" t="inlineStr"/>
@@ -2649,7 +2745,7 @@
       <c r="CO9" s="3" t="inlineStr"/>
       <c r="CP9" s="3" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>-1.5 (-1.5)</t>
         </is>
       </c>
       <c r="CQ9" s="3" t="inlineStr"/>
@@ -2657,7 +2753,7 @@
       <c r="CS9" s="3" t="inlineStr"/>
       <c r="CT9" s="3" t="inlineStr">
         <is>
-          <t>0.5</t>
+          <t>-1.5</t>
         </is>
       </c>
       <c r="CU9" s="3" t="inlineStr"/>
@@ -2867,7 +2963,7 @@
       <c r="CP10" s="3" t="inlineStr"/>
       <c r="CQ10" s="3" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>-1 (-1.5)</t>
         </is>
       </c>
       <c r="CR10" s="3" t="inlineStr"/>
@@ -2875,7 +2971,7 @@
       <c r="CT10" s="3" t="inlineStr"/>
       <c r="CU10" s="3" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>-0.75</t>
         </is>
       </c>
       <c r="CV10" s="3" t="inlineStr"/>
@@ -3085,7 +3181,7 @@
       <c r="CQ11" s="3" t="inlineStr"/>
       <c r="CR11" s="3" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>-1.25 (-1)</t>
         </is>
       </c>
       <c r="CS11" s="3" t="inlineStr"/>
@@ -3093,7 +3189,7 @@
       <c r="CU11" s="3" t="inlineStr"/>
       <c r="CV11" s="3" t="inlineStr">
         <is>
-          <t>0.25 (-1)</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="CW11" s="3" t="inlineStr"/>
@@ -3303,7 +3399,7 @@
       <c r="CR12" s="3" t="inlineStr"/>
       <c r="CS12" s="3" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>-1.25 (-1.25)</t>
         </is>
       </c>
       <c r="CT12" s="3" t="inlineStr"/>
@@ -3311,7 +3407,7 @@
       <c r="CV12" s="3" t="inlineStr"/>
       <c r="CW12" s="3" t="inlineStr">
         <is>
-          <t>0.25</t>
+          <t>-0.75</t>
         </is>
       </c>
       <c r="CX12" s="3" t="inlineStr"/>
@@ -3513,7 +3609,7 @@
       <c r="CO13" s="3" t="inlineStr"/>
       <c r="CP13" s="3" t="inlineStr">
         <is>
-          <t>-0.25</t>
+          <t>-0.25 (-1.25)</t>
         </is>
       </c>
       <c r="CQ13" s="3" t="inlineStr"/>
@@ -3521,7 +3617,7 @@
       <c r="CS13" s="3" t="inlineStr"/>
       <c r="CT13" s="3" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>-0.5 (-1)</t>
         </is>
       </c>
       <c r="CU13" s="3" t="inlineStr"/>
@@ -3529,7 +3625,7 @@
       <c r="CW13" s="3" t="inlineStr"/>
       <c r="CX13" s="3" t="inlineStr">
         <is>
-          <t>0.25</t>
+          <t>-0.25</t>
         </is>
       </c>
       <c r="CY13" s="3" t="inlineStr"/>

</xml_diff>

<commit_message>
Mise à jour des projections des banques centrales (2026-09-19)
</commit_message>
<xml_diff>
--- a/data/boe/boe_mpr.xlsx
+++ b/data/boe/boe_mpr.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet name="Résumé (Table 1.A)" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Scénarios" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -90,7 +91,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -102,6 +103,7 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -467,7 +469,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U19"/>
+  <dimension ref="A1:U21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -2125,15 +2127,69 @@
         </is>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>2026-04</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr"/>
+      <c r="C17" s="3" t="inlineStr"/>
+      <c r="D17" s="3" t="inlineStr"/>
+      <c r="E17" s="3" t="inlineStr"/>
+      <c r="F17" s="3" t="inlineStr"/>
+      <c r="G17" s="3" t="inlineStr"/>
+      <c r="H17" s="3" t="inlineStr"/>
+      <c r="I17" s="3" t="inlineStr"/>
+      <c r="J17" s="3" t="inlineStr"/>
+      <c r="K17" s="3" t="inlineStr"/>
+      <c r="L17" s="3" t="inlineStr"/>
+      <c r="M17" s="3" t="inlineStr"/>
+      <c r="N17" s="3" t="inlineStr"/>
+      <c r="O17" s="3" t="inlineStr"/>
+      <c r="P17" s="3" t="inlineStr"/>
+      <c r="Q17" s="3" t="inlineStr"/>
+      <c r="R17" s="3" t="inlineStr"/>
+      <c r="S17" s="3" t="inlineStr"/>
+      <c r="T17" s="3" t="inlineStr"/>
+      <c r="U17" s="3" t="inlineStr"/>
+    </row>
     <row r="18">
-      <c r="A18" s="4" t="inlineStr">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr"/>
+      <c r="C18" s="3" t="inlineStr"/>
+      <c r="D18" s="3" t="inlineStr"/>
+      <c r="E18" s="3" t="inlineStr"/>
+      <c r="F18" s="3" t="inlineStr"/>
+      <c r="G18" s="3" t="inlineStr"/>
+      <c r="H18" s="3" t="inlineStr"/>
+      <c r="I18" s="3" t="inlineStr"/>
+      <c r="J18" s="3" t="inlineStr"/>
+      <c r="K18" s="3" t="inlineStr"/>
+      <c r="L18" s="3" t="inlineStr"/>
+      <c r="M18" s="3" t="inlineStr"/>
+      <c r="N18" s="3" t="inlineStr"/>
+      <c r="O18" s="3" t="inlineStr"/>
+      <c r="P18" s="3" t="inlineStr"/>
+      <c r="Q18" s="3" t="inlineStr"/>
+      <c r="R18" s="3" t="inlineStr"/>
+      <c r="S18" s="3" t="inlineStr"/>
+      <c r="T18" s="3" t="inlineStr"/>
+      <c r="U18" s="3" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
         <is>
           <t>Colonnes alignées par horizon (année en cours, +1, +2, +3), pas par trimestre calendaire : chaque rapport MPR utilise un trimestre de référence différent selon son mois de publication (ex: rapport de février -&gt; Q1, rapport de novembre -&gt; Q4). Le trimestre exact de chaque valeur est rappelé entre crochets.</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="4" t="inlineStr">
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
         <is>
           <t>* Bank Rate : chemin implicite par les marchés sur lequel les projections sont conditionnées (la BoE ne prévoit pas sa propre trajectoire de taux).</t>
         </is>
@@ -2150,4 +2206,1070 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G30"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Date du MPR</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Scénario</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Variable</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Année en cours</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Année +1</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Année +2</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Année +3</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="5" t="inlineStr">
+        <is>
+          <t>2026-04</t>
+        </is>
+      </c>
+      <c r="B2" s="5" t="inlineStr">
+        <is>
+          <t>Scenario A</t>
+        </is>
+      </c>
+      <c r="C2" s="5" t="inlineStr">
+        <is>
+          <t>Inflation IPC</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>[2026 Q2] 3.1</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>[2027 Q2] 2.9</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>[2028 Q2] 1.5</t>
+        </is>
+      </c>
+      <c r="G2" s="3" t="inlineStr">
+        <is>
+          <t>[2029 Q2] 1.7</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>2026-04</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>Scenario A</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>PIB (glissement annuel)</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>[2026 Q2] 0.7</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>[2027 Q2] 0.8</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>[2028 Q2] 1.7</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>[2029 Q2] 1.8</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>2026-04</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>Scenario A</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>Écart de production</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>[2026 Q2] -1.1</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>[2027 Q2] -1.5</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>[2028 Q2] -1.0</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>[2029 Q2] -0.8</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>2026-04</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>Scenario A</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>Taux de chômage</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>[2026 Q2] 5.1</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>[2027 Q2] 5.5</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>[2028 Q2] 5.4</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>[2029 Q2] 5.1</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>2026-04</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>Scenario B</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>Inflation IPC</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>[2026 Q2] 3.1</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>[2027 Q2] 3.2</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>[2028 Q2] 2.0</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="inlineStr">
+        <is>
+          <t>[2029 Q2] 2.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>2026-04</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>Scenario B</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>PIB (glissement annuel)</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>[2026 Q2] 0.7</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>[2027 Q2] 0.8</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>[2028 Q2] 1.7</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>[2029 Q2] 1.7</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>2026-04</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>Scenario B</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>Écart de production</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>[2026 Q2] -1.1</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>[2027 Q2] -1.4</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>[2028 Q2] -1.0</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="inlineStr">
+        <is>
+          <t>[2029 Q2] -0.8</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>2026-04</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>Scenario B</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>Taux de chômage</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>[2026 Q2] 5.1</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>[2027 Q2] 5.5</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>[2028 Q2] 5.4</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>[2029 Q2] 5.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>2026-04</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>Scenario C</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>Inflation IPC</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>[2026 Q2] 3.6</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>[2027 Q2] 5.6</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>[2028 Q2] 2.9</t>
+        </is>
+      </c>
+      <c r="G10" s="3" t="inlineStr">
+        <is>
+          <t>[2029 Q2] 2.6</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>2026-04</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>Scenario C</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>PIB (glissement annuel)</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>[2026 Q2] 0.7</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>[2027 Q2] 0.5</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>[2028 Q2] 1.7</t>
+        </is>
+      </c>
+      <c r="G11" s="3" t="inlineStr">
+        <is>
+          <t>[2029 Q2] 1.8</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>2026-04</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>Scenario C</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>Écart de production</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>[2026 Q2] -1.1</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>[2027 Q2] -1.7</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>[2028 Q2] -1.3</t>
+        </is>
+      </c>
+      <c r="G12" s="3" t="inlineStr">
+        <is>
+          <t>[2029 Q2] -1.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>2026-04</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>Scenario C</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>Taux de chômage</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>[2026 Q2] 5.1</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>[2027 Q2] 5.6</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>[2028 Q2] 5.6</t>
+        </is>
+      </c>
+      <c r="G13" s="3" t="inlineStr">
+        <is>
+          <t>[2029 Q2] 5.3</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>Adverse scenario</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>Inflation IPC</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>[2026 Q3] 3.1</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>[2027 Q3] 4.1</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>[2028 Q3] 2.8</t>
+        </is>
+      </c>
+      <c r="G14" s="3" t="inlineStr">
+        <is>
+          <t>[2029 Q3] 2.4</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>Adverse scenario</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>PIB (glissement annuel)</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>[2026 Q3] 1.1</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>[2027 Q3] 0.9</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>[2028 Q3] 1.6</t>
+        </is>
+      </c>
+      <c r="G15" s="3" t="inlineStr">
+        <is>
+          <t>[2029 Q3] 1.7</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>Adverse scenario</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>Écart de production</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>[2026 Q3] -1.1</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>[2027 Q3] -1.2</t>
+        </is>
+      </c>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>[2028 Q3] -1.0</t>
+        </is>
+      </c>
+      <c r="G16" s="3" t="inlineStr">
+        <is>
+          <t>[2029 Q3] -0.9</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>Adverse scenario</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>Taux de chômage</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>[2026 Q3] 5.0</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>[2027 Q3] 5.5</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t>[2028 Q3] 5.4</t>
+        </is>
+      </c>
+      <c r="G17" s="3" t="inlineStr">
+        <is>
+          <t>[2029 Q3] 5.3</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>Adverse scenario</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>Bank Rate (implicite marchés)*</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>[2026 Q3] 3.8</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="inlineStr">
+        <is>
+          <t>[2027 Q3] 4.2</t>
+        </is>
+      </c>
+      <c r="F18" s="3" t="inlineStr">
+        <is>
+          <t>[2028 Q3] 4.2</t>
+        </is>
+      </c>
+      <c r="G18" s="3" t="inlineStr">
+        <is>
+          <t>[2029 Q3] 4.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>Central projection</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>Inflation IPC</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>[2026 Q3] 2.9</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>[2027 Q3] 2.6</t>
+        </is>
+      </c>
+      <c r="F19" s="3" t="inlineStr">
+        <is>
+          <t>[2028 Q3] 1.8</t>
+        </is>
+      </c>
+      <c r="G19" s="3" t="inlineStr">
+        <is>
+          <t>[2029 Q3] 1.9</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>Central projection</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>PIB (glissement annuel)</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>[2026 Q3] 1.1</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="inlineStr">
+        <is>
+          <t>[2027 Q3] 1.1</t>
+        </is>
+      </c>
+      <c r="F20" s="3" t="inlineStr">
+        <is>
+          <t>[2028 Q3] 1.7</t>
+        </is>
+      </c>
+      <c r="G20" s="3" t="inlineStr">
+        <is>
+          <t>[2029 Q3] 1.6</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>Central projection</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>Écart de production</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>[2026 Q3] -1.1</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="inlineStr">
+        <is>
+          <t>[2027 Q3] -1.0</t>
+        </is>
+      </c>
+      <c r="F21" s="3" t="inlineStr">
+        <is>
+          <t>[2028 Q3] -0.7</t>
+        </is>
+      </c>
+      <c r="G21" s="3" t="inlineStr">
+        <is>
+          <t>[2029 Q3] -0.6</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>Central projection</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>Taux de chômage</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>[2026 Q3] 5.0</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="inlineStr">
+        <is>
+          <t>[2027 Q3] 5.3</t>
+        </is>
+      </c>
+      <c r="F22" s="3" t="inlineStr">
+        <is>
+          <t>[2028 Q3] 5.2</t>
+        </is>
+      </c>
+      <c r="G22" s="3" t="inlineStr">
+        <is>
+          <t>[2029 Q3] 5.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t>Central projection</t>
+        </is>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>Bank Rate (implicite marchés)*</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>[2026 Q3] 3.8</t>
+        </is>
+      </c>
+      <c r="E23" s="3" t="inlineStr">
+        <is>
+          <t>[2027 Q3] 4.2</t>
+        </is>
+      </c>
+      <c r="F23" s="3" t="inlineStr">
+        <is>
+          <t>[2028 Q3] 4.2</t>
+        </is>
+      </c>
+      <c r="G23" s="3" t="inlineStr">
+        <is>
+          <t>[2029 Q3] 4.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="inlineStr">
+        <is>
+          <t>Milder scenario</t>
+        </is>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>Inflation IPC</t>
+        </is>
+      </c>
+      <c r="D24" s="3" t="inlineStr">
+        <is>
+          <t>[2026 Q3] 2.7</t>
+        </is>
+      </c>
+      <c r="E24" s="3" t="inlineStr">
+        <is>
+          <t>[2027 Q3] 2.4</t>
+        </is>
+      </c>
+      <c r="F24" s="3" t="inlineStr">
+        <is>
+          <t>[2028 Q3] 1.7</t>
+        </is>
+      </c>
+      <c r="G24" s="3" t="inlineStr">
+        <is>
+          <t>[2029 Q3] 1.7</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="inlineStr">
+        <is>
+          <t>Milder scenario</t>
+        </is>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>PIB (glissement annuel)</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t>[2026 Q3] 1.1</t>
+        </is>
+      </c>
+      <c r="E25" s="3" t="inlineStr">
+        <is>
+          <t>[2027 Q3] 1.1</t>
+        </is>
+      </c>
+      <c r="F25" s="3" t="inlineStr">
+        <is>
+          <t>[2028 Q3] 1.6</t>
+        </is>
+      </c>
+      <c r="G25" s="3" t="inlineStr">
+        <is>
+          <t>[2029 Q3] 1.6</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="inlineStr">
+        <is>
+          <t>Milder scenario</t>
+        </is>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>Écart de production</t>
+        </is>
+      </c>
+      <c r="D26" s="3" t="inlineStr">
+        <is>
+          <t>[2026 Q3] -1.2</t>
+        </is>
+      </c>
+      <c r="E26" s="3" t="inlineStr">
+        <is>
+          <t>[2027 Q3] -1.1</t>
+        </is>
+      </c>
+      <c r="F26" s="3" t="inlineStr">
+        <is>
+          <t>[2028 Q3] -0.9</t>
+        </is>
+      </c>
+      <c r="G26" s="3" t="inlineStr">
+        <is>
+          <t>[2029 Q3] -0.8</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="inlineStr">
+        <is>
+          <t>Milder scenario</t>
+        </is>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>Taux de chômage</t>
+        </is>
+      </c>
+      <c r="D27" s="3" t="inlineStr">
+        <is>
+          <t>[2026 Q3] 5.0</t>
+        </is>
+      </c>
+      <c r="E27" s="3" t="inlineStr">
+        <is>
+          <t>[2027 Q3] 5.5</t>
+        </is>
+      </c>
+      <c r="F27" s="3" t="inlineStr">
+        <is>
+          <t>[2028 Q3] 5.3</t>
+        </is>
+      </c>
+      <c r="G27" s="3" t="inlineStr">
+        <is>
+          <t>[2029 Q3] 5.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="inlineStr">
+        <is>
+          <t>Milder scenario</t>
+        </is>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>Bank Rate (implicite marchés)*</t>
+        </is>
+      </c>
+      <c r="D28" s="3" t="inlineStr">
+        <is>
+          <t>[2026 Q3] 3.8</t>
+        </is>
+      </c>
+      <c r="E28" s="3" t="inlineStr">
+        <is>
+          <t>[2027 Q3] 4.2</t>
+        </is>
+      </c>
+      <c r="F28" s="3" t="inlineStr">
+        <is>
+          <t>[2028 Q3] 4.2</t>
+        </is>
+      </c>
+      <c r="G28" s="3" t="inlineStr">
+        <is>
+          <t>[2029 Q3] 4.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>Certaines éditions (ex: avril et juillet 2026) présentent plusieurs scénarios au lieu d'une projection centrale unique, tous conditionnés sur le même chemin de Bank Rate implicite par les marchés -- pas de comparaison avec le rapport précédent dans ce format.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>